<commit_message>
No oil shale 2035 scenario
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_no_oil_shale_2035.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_no_oil_shale_2035.xlsx
@@ -8,24 +8,35 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2C795C1-E01F-48BC-BF51-A303A0BBB049}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3728C0C9-49AE-4DC2-AAEE-BD26567F9E0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="constraint" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>pset_ci</t>
   </si>
@@ -33,73 +44,52 @@
     <t>EST</t>
   </si>
   <si>
-    <t>~TFM_INS-TS</t>
-  </si>
-  <si>
-    <t>attribute</t>
-  </si>
-  <si>
-    <t>pset_set</t>
-  </si>
-  <si>
-    <t>process</t>
-  </si>
-  <si>
-    <t>attrib_cond</t>
-  </si>
-  <si>
-    <t>limtype</t>
-  </si>
-  <si>
-    <t>other_indexes</t>
-  </si>
-  <si>
-    <t>commodity</t>
-  </si>
-  <si>
-    <t>region</t>
-  </si>
-  <si>
-    <t>rcap_bnd</t>
-  </si>
-  <si>
-    <t>ep_*</t>
-  </si>
-  <si>
-    <t>up</t>
-  </si>
-  <si>
-    <t>coal</t>
+    <t>~UC_Sets: R_E: AllRegions</t>
+  </si>
+  <si>
+    <t>~UC_T:UC_RHSRT</t>
+  </si>
+  <si>
+    <t>UC_N</t>
+  </si>
+  <si>
+    <t>Pset_Set</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>LimType</t>
+  </si>
+  <si>
+    <t>UC_CAP</t>
+  </si>
+  <si>
+    <t>UC_RHSRT~0</t>
+  </si>
+  <si>
+    <t>UC_Desc</t>
+  </si>
+  <si>
+    <t>UC_max_oil_shale_capacity</t>
+  </si>
+  <si>
+    <t>Subcritical Coal,Supercritical Coal</t>
+  </si>
+  <si>
+    <t>UP</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="186"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="186"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -117,7 +107,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -125,39 +115,15 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thick">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.39997558519241921"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="2"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="3">
-    <cellStyle name="Heading 2" xfId="1" builtinId="17"/>
-    <cellStyle name="Heading 3" xfId="2" builtinId="18"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -436,85 +402,79 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B3:M6"/>
+  <dimension ref="B5:J9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="2" max="2" width="25.85546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.85546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="16.140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11.140625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="11.140625" customWidth="1"/>
+    <col min="9" max="9" width="12" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:13" ht="18" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="2" t="s">
+    <row r="5" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="2:13" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="3" t="s">
+    <row r="7" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="E7" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="3" t="s">
+    </row>
+    <row r="8" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="C8" t="s">
+        <v>5</v>
+      </c>
+      <c r="D8" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E8" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F8" t="s">
+        <v>7</v>
+      </c>
+      <c r="G8" t="s">
+        <v>8</v>
+      </c>
+      <c r="H8" t="s">
+        <v>1</v>
+      </c>
+      <c r="I8" t="s">
+        <v>9</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E9">
+        <v>2035</v>
+      </c>
+      <c r="F9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G9">
+        <v>1</v>
+      </c>
+      <c r="H9">
+        <v>0</v>
+      </c>
+      <c r="I9">
         <v>5</v>
       </c>
-      <c r="F4" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="H4" s="3">
-        <v>0</v>
-      </c>
-      <c r="I4" s="3">
-        <v>2022</v>
-      </c>
-      <c r="J4" s="3">
-        <v>2035</v>
-      </c>
-      <c r="K4" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="L4" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="M4" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="5" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D5" t="s">
-        <v>14</v>
-      </c>
-      <c r="E5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G5" t="s">
-        <v>1</v>
-      </c>
-      <c r="H5">
-        <v>4</v>
-      </c>
-      <c r="J5">
-        <v>0</v>
-      </c>
-      <c r="K5" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="6" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
-      <c r="K6" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Oil shale ban 2035
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_no_oil_shale_2035.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_no_oil_shale_2035.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3728C0C9-49AE-4DC2-AAEE-BD26567F9E0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DE2CBD8-AD01-465E-B310-6D8C72B6540C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,67 +36,55 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>pset_ci</t>
   </si>
   <si>
-    <t>EST</t>
-  </si>
-  <si>
     <t>~UC_Sets: R_E: AllRegions</t>
   </si>
   <si>
-    <t>~UC_T:UC_RHSRT</t>
-  </si>
-  <si>
     <t>UC_N</t>
   </si>
   <si>
     <t>Pset_Set</t>
   </si>
   <si>
-    <t>Year</t>
-  </si>
-  <si>
-    <t>LimType</t>
-  </si>
-  <si>
     <t>UC_CAP</t>
   </si>
   <si>
     <t>UC_RHSRT~0</t>
   </si>
   <si>
-    <t>UC_Desc</t>
-  </si>
-  <si>
     <t>UC_max_oil_shale_capacity</t>
   </si>
   <si>
     <t>Subcritical Coal,Supercritical Coal</t>
   </si>
   <si>
-    <t>UP</t>
+    <t>pset_co</t>
+  </si>
+  <si>
+    <t>UC_ACT</t>
+  </si>
+  <si>
+    <t>UC_RHSRT</t>
+  </si>
+  <si>
+    <t>~UC_T:</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="186"/>
     </font>
   </fonts>
   <fills count="2">
@@ -119,9 +107,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -402,77 +389,75 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B5:J9"/>
+  <dimension ref="B5:K9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="25.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.140625" customWidth="1"/>
-    <col min="9" max="9" width="12" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.85546875" customWidth="1"/>
+    <col min="6" max="6" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.140625" customWidth="1"/>
+    <col min="10" max="11" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="5" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
         <v>2</v>
       </c>
+      <c r="C8" t="s">
+        <v>3</v>
+      </c>
+      <c r="D8" t="s">
+        <v>0</v>
+      </c>
+      <c r="E8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+      <c r="G8" t="s">
+        <v>4</v>
+      </c>
+      <c r="H8">
+        <v>2022</v>
+      </c>
+      <c r="I8">
+        <v>2035</v>
+      </c>
+      <c r="J8" t="s">
+        <v>10</v>
+      </c>
+      <c r="K8" t="s">
+        <v>5</v>
+      </c>
     </row>
-    <row r="7" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="E7" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="8" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B8" t="s">
-        <v>4</v>
-      </c>
-      <c r="C8" t="s">
-        <v>5</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="E8" s="1" t="s">
+    <row r="9" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
         <v>6</v>
       </c>
-      <c r="F8" t="s">
+      <c r="C9" t="s">
         <v>7</v>
-      </c>
-      <c r="G8" t="s">
-        <v>8</v>
-      </c>
-      <c r="H8" t="s">
-        <v>1</v>
-      </c>
-      <c r="I8" t="s">
-        <v>9</v>
-      </c>
-      <c r="J8" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="9" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B9" t="s">
-        <v>11</v>
-      </c>
-      <c r="C9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E9">
-        <v>2035</v>
-      </c>
-      <c r="F9" t="s">
-        <v>13</v>
       </c>
       <c r="G9">
         <v>1</v>
       </c>
-      <c r="H9">
+      <c r="I9">
         <v>0</v>
       </c>
-      <c r="I9">
+      <c r="K9">
         <v>5</v>
       </c>
     </row>

</xml_diff>